<commit_message>
Add Google Sheets order integration
Orders POST to a Google Apps Script web app (works on serverless),
with local Excel fallback for dev. Includes setup script + env example.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/orders.xlsx
+++ b/data/orders.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:K6"/>
+  <dimension ref="A1:K4"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -506,25 +506,25 @@
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>MM-260628-M8UO</v>
+        <v>MM-260628-A98B</v>
       </c>
       <c r="B4" t="str">
-        <v>2026-06-27T23:42:11.838Z</v>
+        <v>2026-06-27T23:44:10.040Z</v>
       </c>
       <c r="C4" t="str">
         <v>جديد</v>
       </c>
       <c r="D4" t="str">
-        <v>raccc</v>
+        <v>eeeee</v>
       </c>
       <c r="E4" t="str">
-        <v>0600000000</v>
+        <v>0700000000</v>
       </c>
       <c r="F4" t="str">
-        <v>c</v>
+        <v>rrrrrr</v>
       </c>
       <c r="G4" t="str">
-        <v>casssssssss</v>
+        <v>rrrrrrrrr</v>
       </c>
       <c r="H4" t="str">
         <v>مصباح شمسي ذكي على شكل كاميرا</v>
@@ -537,81 +537,11 @@
       </c>
       <c r="K4">
         <v>150</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="str">
-        <v>MM-260628-A98B</v>
-      </c>
-      <c r="B5" t="str">
-        <v>2026-06-27T23:44:10.040Z</v>
-      </c>
-      <c r="C5" t="str">
-        <v>جديد</v>
-      </c>
-      <c r="D5" t="str">
-        <v>eeeee</v>
-      </c>
-      <c r="E5" t="str">
-        <v>0700000000</v>
-      </c>
-      <c r="F5" t="str">
-        <v>rrrrrr</v>
-      </c>
-      <c r="G5" t="str">
-        <v>rrrrrrrrr</v>
-      </c>
-      <c r="H5" t="str">
-        <v>مصباح شمسي ذكي على شكل كاميرا</v>
-      </c>
-      <c r="I5" t="str">
-        <v>solar-camera-security-light</v>
-      </c>
-      <c r="J5">
-        <v>1</v>
-      </c>
-      <c r="K5">
-        <v>150</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="str">
-        <v>MM-260628-8V54</v>
-      </c>
-      <c r="B6" t="str">
-        <v>2026-06-28T10:21:30.098Z</v>
-      </c>
-      <c r="C6" t="str">
-        <v>جديد</v>
-      </c>
-      <c r="D6" t="str">
-        <v>ttttttt</v>
-      </c>
-      <c r="E6" t="str">
-        <v>0600000000</v>
-      </c>
-      <c r="F6" t="str">
-        <v>ttttttt</v>
-      </c>
-      <c r="G6" t="str">
-        <v>ttttttttt</v>
-      </c>
-      <c r="H6" t="str">
-        <v>نشار الملابس المعدني 4 طبقات</v>
-      </c>
-      <c r="I6" t="str">
-        <v>metal-clothes-hanger-4-tier</v>
-      </c>
-      <c r="J6">
-        <v>1</v>
-      </c>
-      <c r="K6">
-        <v>240</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:K6"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:K4"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>